<commit_message>
Edited the Building data schematics and added data into database
</commit_message>
<xml_diff>
--- a/Ice Depth Project/Source_Documents - Items to be copied/billing_data/BillHistory_Account_Electric.xlsx
+++ b/Ice Depth Project/Source_Documents - Items to be copied/billing_data/BillHistory_Account_Electric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\other-files\school\database_dev\The-Windigo-Data-Team-Summer-2026\Ice Depth Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\other-files\school\database_dev\The-Windigo-Data-Team-Summer-2026\Ice Depth Project\Source_Documents - Items to be copied\billing_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DEBDD70-01CA-441F-BF0B-52A4B72FE506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F00BB91-C365-4880-BD5E-7DD549515BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2C695120-188F-48AA-88E0-ADAA39F614CF}"/>
+    <workbookView xWindow="38280" yWindow="690" windowWidth="29040" windowHeight="17520" xr2:uid="{2C695120-188F-48AA-88E0-ADAA39F614CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -663,31 +663,31 @@
       <c r="C2">
         <v>30</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>1932.48</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>1948.2</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>2451.59</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
         <v>749.25</v>
       </c>
       <c r="H2">
         <v>60</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="2">
         <v>162.47</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="2">
         <v>363.51</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
         <v>0</v>
       </c>
       <c r="M2">
@@ -745,31 +745,31 @@
       <c r="C3">
         <v>28</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>2028.43</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>1989</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>2632.44</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
         <v>749.25</v>
       </c>
       <c r="H3">
         <v>56</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="2">
         <v>166.39</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>379.39</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="2">
         <v>74.44</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="2">
         <v>7814.65</v>
       </c>
       <c r="M3">
@@ -827,31 +827,31 @@
       <c r="C4">
         <v>33</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>2137.66</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>2184.9</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>2250.64</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="2">
         <v>627.75</v>
       </c>
       <c r="H4">
         <v>66</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="2">
         <v>177.18</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>370.52</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
         <v>0</v>
       </c>
       <c r="M4">
@@ -909,31 +909,31 @@
       <c r="C5">
         <v>29</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>2246.69</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="2">
         <v>2230.38</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>2331.02</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="2">
         <v>627.75</v>
       </c>
       <c r="H5">
         <v>58</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="2">
         <v>181.79</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>382.1</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
         <v>0</v>
       </c>
       <c r="M5">
@@ -991,31 +991,31 @@
       <c r="C6">
         <v>27</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>3380.43</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>3367.38</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>3717.58</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="2">
         <v>627.75</v>
       </c>
       <c r="H6">
         <v>54</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="2">
         <v>256.97000000000003</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>568.52</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="2">
         <v>84.53</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="2">
         <v>8869.6200000000008</v>
       </c>
       <c r="M6">
@@ -1073,31 +1073,31 @@
       <c r="C7">
         <v>35</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>2298.6799999999998</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>2687.89</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>2634.61</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="2">
         <v>559.94000000000005</v>
       </c>
       <c r="H7">
         <v>70</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="2">
         <v>124.36</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <v>417.09</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="2">
         <v>77.05</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="2">
         <v>0</v>
       </c>
       <c r="M7">
@@ -1155,31 +1155,31 @@
       <c r="C8">
         <v>34</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>2196.42</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>2514.67</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <v>2302.6799999999998</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="2">
         <v>555.24</v>
       </c>
       <c r="H8">
         <v>68</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="2">
         <v>68.16</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="2">
         <v>383.57</v>
       </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
         <v>0</v>
       </c>
       <c r="M8">
@@ -1237,31 +1237,31 @@
       <c r="C9">
         <v>28</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>1772.36</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>1872.91</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <v>2125.5500000000002</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="2">
         <v>555.24</v>
       </c>
       <c r="H9">
         <v>56</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="2">
         <v>60.59</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="2">
         <v>320.45</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="2">
         <v>66.59</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="2">
         <v>6990.56</v>
       </c>
       <c r="M9">
@@ -1319,31 +1319,31 @@
       <c r="C10">
         <v>28</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>2103.0500000000002</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>2056.48</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <v>3267.05</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="2">
         <v>555.24</v>
       </c>
       <c r="H10">
         <v>56</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="2">
         <v>-1378.54</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="2">
         <v>331.28</v>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
+      <c r="K10" s="2">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
         <v>0</v>
       </c>
       <c r="M10">
@@ -1401,31 +1401,31 @@
       <c r="C11">
         <v>30</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>2199.02</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>1990.19</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
         <v>2755.34</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="2">
         <v>518.89</v>
       </c>
       <c r="H11">
         <v>60</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="2">
         <v>-754.22</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="2">
         <v>336.78</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="2">
         <v>74.81</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="2">
         <v>0</v>
       </c>
       <c r="M11">
@@ -1483,31 +1483,31 @@
       <c r="C12">
         <v>30</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>2217.85</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>1846.35</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="2">
         <v>2775.02</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="2">
         <v>518.89</v>
       </c>
       <c r="H12">
         <v>60</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="2">
         <v>62.84</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="2">
         <v>372.36</v>
       </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
+      <c r="K12" s="2">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
         <v>0</v>
       </c>
       <c r="M12">
@@ -1565,31 +1565,31 @@
       <c r="C13">
         <v>32</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="2">
         <v>2135.9699999999998</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="2">
         <v>2151.33</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="2">
         <v>2873.43</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="2">
         <v>518.89</v>
       </c>
       <c r="H13">
         <v>64</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="2">
         <v>64.55</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="2">
         <v>388.75</v>
       </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
         <v>0</v>
       </c>
       <c r="M13">
@@ -1647,31 +1647,31 @@
       <c r="C14">
         <v>31</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="2">
         <v>1812.37</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="2">
         <v>1711</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="2">
         <v>2125.5500000000002</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="2">
         <v>482.53</v>
       </c>
       <c r="H14">
         <v>62</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="2">
         <v>58.98</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="2">
         <v>310.99</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="2">
         <v>59.59</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="2">
         <v>6255.27</v>
       </c>
       <c r="M14">
@@ -1729,31 +1729,31 @@
       <c r="C15">
         <v>31</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>1562.13</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="2">
         <v>1786.23</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="2">
         <v>2007.46</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="2">
         <v>482.53</v>
       </c>
       <c r="H15">
         <v>62</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="2">
         <v>58.61</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="2">
         <v>296.31</v>
       </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
+      <c r="K15" s="2">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
         <v>0</v>
       </c>
       <c r="M15">

</xml_diff>